<commit_message>
added sebi informal guidance to parsing agent
</commit_message>
<xml_diff>
--- a/Pravartiya/data/test.xlsx
+++ b/Pravartiya/data/test.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Verticals</t>
   </si>
@@ -46,40 +46,25 @@
     <t>SEBI</t>
   </si>
   <si>
-    <t>Regulations</t>
-  </si>
-  <si>
-    <t>January</t>
-  </si>
-  <si>
-    <t>2026-01-22</t>
-  </si>
-  <si>
-    <t>Securities and Exchange Board of India (Listing Obligations and Disclosure Requirements) Regulations, 2015 [Last amended on January 22, 2026]</t>
-  </si>
-  <si>
-    <t>https://www.sebi.gov.in/sebi_data/attachdocs/apr-2026/1777351317428.pdf</t>
-  </si>
-  <si>
-    <t>Securities_and_Exchange_Board_of_India_Listing_Obligations_and_Disclosure_Requir_500e67fd.pdf</t>
-  </si>
-  <si>
-    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Regulations/2026/January/Securities_and_Exchange_Board_of_India_Listing_Obligations_and_Disclosure_Requir_500e67fd.pdf</t>
-  </si>
-  <si>
-    <t>Securities and Exchange Board of India (Listing Obligations and Disclosure Requirements) (Amendment) Regulations, 2026</t>
-  </si>
-  <si>
-    <t>https://www.sebi.gov.in/sebi_data/attachdocs/jan-2026/1769600297568.pdf</t>
-  </si>
-  <si>
-    <t>Securities_and_Exchange_Board_of_India_Listing_Obligations_and_Disclosure_Requir_d9dfa16a.pdf</t>
-  </si>
-  <si>
-    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Regulations/2026/January/Securities_and_Exchange_Board_of_India_Listing_Obligations_and_Disclosure_Requir_d9dfa16a.pdf</t>
-  </si>
-  <si>
-    <t/>
+    <t>Informal Guidance</t>
+  </si>
+  <si>
+    <t>February</t>
+  </si>
+  <si>
+    <t>2026-02-06</t>
+  </si>
+  <si>
+    <t>Request for Informal Guidance by way of an interpretative letter under the Securities and Exchange Board of India (Informal Guidance) Scheme, 2025 received from Punjab National Bank seeking interpretation of the provisions of Regulation 27 of the SEBI (Listing Obligations and Disclosure Requirements) Regulations, 2015 and SEBI Circular for implementation of recommendations of the Expert Committee for facilitating ease of doing business for listed entities dated 31.12.2024</t>
+  </si>
+  <si>
+    <t>https://www.sebi.gov.in/sebi_data/commondocs/feb-2026/PNB%20-%20Informal%20Guidance%20Letter%20by%20SEBI_p.pdf</t>
+  </si>
+  <si>
+    <t>Request_for_Informal_Guidance_by_way_of_an_interpretative_letter_under_the_Secur_948a270a.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Informal Guidance/2026/February/Request_for_Informal_Guidance_by_way_of_an_interpretative_letter_under_the_Secur_948a270a.pdf</t>
   </si>
 </sst>
 </file>
@@ -104,7 +89,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -158,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -175,20 +160,11 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -498,15 +474,15 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="9" width="82.7192857142857" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="82.7192857142857" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -568,65 +544,31 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="4">
-        <v>2026</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>21</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
       <c r="C4" s="4"/>
-      <c r="D4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>21</v>
-      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
-      <c r="C5" s="8"/>
+      <c r="C5" s="4"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -637,7 +579,7 @@
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
-      <c r="C6" s="8"/>
+      <c r="C6" s="4"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -648,7 +590,7 @@
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
-      <c r="C7" s="8"/>
+      <c r="C7" s="4"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>

</xml_diff>

<commit_message>
nse bse code updated, till here we have finalised Informal Guidance,Press Release,Consultation Paper,Master Circular
</commit_message>
<xml_diff>
--- a/Pravartiya/data/test.xlsx
+++ b/Pravartiya/data/test.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
   <si>
     <t>Verticals</t>
   </si>
@@ -43,100 +43,55 @@
     <t>Path</t>
   </si>
   <si>
-    <t>SEBI</t>
-  </si>
-  <si>
-    <t>Press Release</t>
-  </si>
-  <si>
-    <t>April</t>
-  </si>
-  <si>
-    <t>2026-04-29</t>
-  </si>
-  <si>
-    <t>SEBI operationalises Past Risk and Return Verification Agency (“PaRRVA”)</t>
-  </si>
-  <si>
-    <t>https://www.sebi.gov.in/sebi_data/attachdocs/apr-2026/1777472194521.pdf</t>
-  </si>
-  <si>
-    <t>SEBI_operationalises_Past_Risk_and_Return_Verification_Agency_PaRRVA_9f11efb2.pdf</t>
-  </si>
-  <si>
-    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Press Release/2026/April/SEBI_operationalises_Past_Risk_and_Return_Verification_Agency_PaRRVA_9f11efb2.pdf</t>
-  </si>
-  <si>
-    <t>2026-04-25</t>
-  </si>
-  <si>
-    <t>SEBI celebrates its 38th Foundation Day</t>
-  </si>
-  <si>
-    <t>https://www.sebi.gov.in/sebi_data/attachdocs/apr-2026/1777116554349.pdf</t>
-  </si>
-  <si>
-    <t>SEBI_celebrates_its_38th_Foundation_Day_aaf0859c.pdf</t>
-  </si>
-  <si>
-    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Press Release/2026/April/SEBI_celebrates_its_38th_Foundation_Day_aaf0859c.pdf</t>
-  </si>
-  <si>
-    <t>2026-04-16</t>
-  </si>
-  <si>
-    <t>Securities and Exchange Board of India (SEBI) signed a Memorandum of Understanding with Financial Intelligence Unit India (FIU-India)</t>
-  </si>
-  <si>
-    <t>https://www.sebi.gov.in/sebi_data/attachdocs/apr-2026/1776340182711.pdf</t>
-  </si>
-  <si>
-    <t>Securities_and_Exchange_Board_of_India_SEBI_signed_a_Memorandum_of_Understanding_e0467cdb.pdf</t>
-  </si>
-  <si>
-    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Press Release/2026/April/Securities_and_Exchange_Board_of_India_SEBI_signed_a_Memorandum_of_Understanding_e0467cdb.pdf</t>
-  </si>
-  <si>
-    <t>2026-04-15</t>
-  </si>
-  <si>
-    <t>Securities and Exchange Board of India (SEBI) signed a Memorandum of Understanding with Department of Telecommunications (DOT), Government of India</t>
-  </si>
-  <si>
-    <t>https://www.sebi.gov.in/sebi_data/attachdocs/apr-2026/1776256038511.pdf</t>
-  </si>
-  <si>
-    <t>Securities_and_Exchange_Board_of_India_SEBI_signed_a_Memorandum_of_Understanding_3fea22f7.pdf</t>
-  </si>
-  <si>
-    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Press Release/2026/April/Securities_and_Exchange_Board_of_India_SEBI_signed_a_Memorandum_of_Understanding_3fea22f7.pdf</t>
-  </si>
-  <si>
-    <t>Shri K.V.R. Murty takes charge as Whole Time Member, SEBI</t>
-  </si>
-  <si>
-    <t>https://www.sebi.gov.in/sebi_data/attachdocs/apr-2026/1776251258103.pdf</t>
-  </si>
-  <si>
-    <t>Shri_K_V_R_Murty_takes_charge_as_Whole_Time_Member_SEBI_72c04e17.pdf</t>
-  </si>
-  <si>
-    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Press Release/2026/April/Shri_K_V_R_Murty_takes_charge_as_Whole_Time_Member_SEBI_72c04e17.pdf</t>
-  </si>
-  <si>
-    <t>2026-04-10</t>
-  </si>
-  <si>
-    <t>Launch of various IT platforms by Chairman, SEBI to improve ease-of-doing business</t>
-  </si>
-  <si>
-    <t>https://www.sebi.gov.in/sebi_data/attachdocs/apr-2026/1775836325260.pdf</t>
-  </si>
-  <si>
-    <t>Launch_of_various_IT_platforms_by_Chairman_SEBI_to_improve_ease_of_doing_busines_5b03b834.pdf</t>
-  </si>
-  <si>
-    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Press Release/2026/April/Launch_of_various_IT_platforms_by_Chairman_SEBI_to_improve_ease_of_doing_busines_5b03b834.pdf</t>
+    <t>Listed Companies</t>
+  </si>
+  <si>
+    <t>Circular-BSE</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>2026-05-04</t>
+  </si>
+  <si>
+    <t>XBRL based filing for Violations related to Code of Conduct (CoC) under SEBI PIT Regulations, 2015</t>
+  </si>
+  <si>
+    <t>https://www.bseindia.com/downloads/UploadDocs/Notices/20260504-17/20260504-17.pdf</t>
+  </si>
+  <si>
+    <t>XBRL_based_filing_for_Violations_related_to_Code_of_Conduct_CoC_under_SEBI_PIT_R_47394cc5.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-BSE/2026/May/XBRL_based_filing_for_Violations_related_to_Code_of_Conduct_CoC_under_SEBI_PIT_R_47394cc5.pdf</t>
+  </si>
+  <si>
+    <t>Circular-NSE</t>
+  </si>
+  <si>
+    <t>XBRL based filing for Violations related to Code of Conduct (CoC) under SEBI (Prohibition of Insider Trading) Regulations, 2015</t>
+  </si>
+  <si>
+    <t>https://nsearchives.nseindia.com//web/circular/2026-05/Violation_of_Code_of_Conduct_20260504201244.pdf</t>
+  </si>
+  <si>
+    <t>XBRL_based_filing_for_Violations_related_to_Code_of_Conduct_CoC_under_SEBI_Prohi_21805baa.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-NSE/2026/May/XBRL_based_filing_for_Violations_related_to_Code_of_Conduct_CoC_under_SEBI_Prohi_21805baa.pdf</t>
+  </si>
+  <si>
+    <t>Filing of disclosures in XBRL format under Regulation 7(2) and Regulation 7(3) of SEBI (Prohibition of Insider Trading) Regulations, 2015</t>
+  </si>
+  <si>
+    <t>https://nsearchives.nseindia.com//web/circular/2026-05/Prohibition_of_Insider_Trading_20260504195923.pdf</t>
+  </si>
+  <si>
+    <t>Filing_of_disclosures_in_XBRL_format_under_Regulation_7_2_and_Regulation_7_3_of_9567ee38.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-NSE/2026/May/Filing_of_disclosures_in_XBRL_format_under_Regulation_7_2_and_Regulation_7_3_of_9567ee38.pdf</t>
   </si>
 </sst>
 </file>
@@ -144,7 +99,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -156,12 +111,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -221,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -238,10 +187,7 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -555,18 +501,18 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="8" width="82.7192857142857" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="82.7192857142857" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -598,7 +544,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
@@ -627,12 +573,12 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C3" s="4">
         <v>2026</v>
@@ -641,7 +587,7 @@
         <v>11</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>18</v>
@@ -661,116 +607,205 @@
         <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="6">
+        <v>17</v>
+      </c>
+      <c r="C4" s="4">
         <v>2026</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I4" s="3" t="s">
-        <v>26</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="6">
-        <v>2026</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>31</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="6">
-        <v>2026</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>35</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="6">
-        <v>2026</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added solution for spacing issue of reference number,added prompt to clean summaries for ppt, till here the regulations summary is bettre, here we dont have mapping to board meeing yet
</commit_message>
<xml_diff>
--- a/Pravartiya/data/test.xlsx
+++ b/Pravartiya/data/test.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
   <si>
     <t>Verticals</t>
   </si>
@@ -46,37 +46,28 @@
     <t>SEBI</t>
   </si>
   <si>
-    <t>Regulations</t>
-  </si>
-  <si>
-    <t>January</t>
-  </si>
-  <si>
-    <t>2026-01-22</t>
-  </si>
-  <si>
-    <t>Securities and Exchange Board of India (Listing Obligations and Disclosure Requirements) Regulations, 2015 [Last amended on January 22, 2026]</t>
-  </si>
-  <si>
-    <t>file:///Users/admin/Downloads/1780915347745.pdf</t>
-  </si>
-  <si>
-    <t>Securities_and_Exchange_Board_of_India_Listing_Obligations_and_Disclosure_Requir_500e67fd.pdf</t>
-  </si>
-  <si>
-    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Regulations/2026/January/Securities_and_Exchange_Board_of_India_Listing_Obligations_and_Disclosure_Requir_500e67fd.pdf</t>
-  </si>
-  <si>
-    <t>Securities and Exchange Board of India (Listing Obligations and Disclosure Requirements) (Amendment) Regulations, 2026</t>
-  </si>
-  <si>
-    <t>https://www.sebi.gov.in/sebi_data/attachdocs/jan-2026/1769600297568.pdf</t>
-  </si>
-  <si>
-    <t>Securities_and_Exchange_Board_of_India_Listing_Obligations_and_Disclosure_Requir_d9dfa16a.pdf</t>
-  </si>
-  <si>
-    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Regulations/2026/January/Securities_and_Exchange_Board_of_India_Listing_Obligations_and_Disclosure_Requir_d9dfa16a.pdf</t>
+    <t>Press Release</t>
+  </si>
+  <si>
+    <t>April</t>
+  </si>
+  <si>
+    <t>2026-04-10</t>
+  </si>
+  <si>
+    <t>Launch of various IT platforms by Chairman, SEBI to improve ease-of-doing business</t>
+  </si>
+  <si>
+    <t>https://www.sebi.gov.in/sebi_data/attachdocs/apr-2026/1775836325260.pdf</t>
+  </si>
+  <si>
+    <t>Launch_of_various_IT_platforms_by_Chairman_SEBI_to_improve_ease_of_doing_busines_5b03b834.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Press Release/2026/April/Launch_of_various_IT_platforms_by_Chairman_SEBI_to_improve_ease_of_doing_busines_5b03b834.pdf</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -155,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -170,6 +161,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
@@ -489,15 +486,15 @@
   <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="105.7192857142857" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="9" width="105.7192857142857" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -559,32 +556,30 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="4">
-        <v>2026</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="A3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>20</v>
+      <c r="B3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>17</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
@@ -616,7 +611,7 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-      <c r="G6" s="6"/>
+      <c r="G6" s="8"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
     </row>
@@ -627,7 +622,7 @@
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="6"/>
+      <c r="G7" s="8"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
     </row>
@@ -759,7 +754,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
-      <c r="G19" s="6"/>
+      <c r="G19" s="8"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
     </row>
@@ -770,7 +765,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
-      <c r="G20" s="6"/>
+      <c r="G20" s="8"/>
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
     </row>

</xml_diff>